<commit_message>
RAG Part A: corpus v2, retrieval fixes, reproducible baseline
</commit_message>
<xml_diff>
--- a/src/evaluators/rag_benchmark_questions.xlsx
+++ b/src/evaluators/rag_benchmark_questions.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K69"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -506,6 +506,11 @@
           <t>notes</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>expected_answer</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -515,7 +520,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>answerable</t>
+          <t>near_miss</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -525,30 +530,26 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>answered</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>no fasting is required; fast for 8 to 12 hours</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>mri</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>may be asked not to eat or drink for 4 to 6 hours before the scan</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>no fasting is required; fast for 8 to 12 hours</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Fasting window is explicit in the MRI page.</t>
+          <t>The NLM-authored MRI replacement gives no fasting instructions or duration.</t>
         </is>
       </c>
     </row>
@@ -580,7 +581,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>does not use ionizing radiation; uses powerful magnets and radio waves</t>
+          <t>does not use x-rays or other radiation; uses magnets, radio waves, and a computer</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
@@ -593,7 +594,12 @@
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Direct contrast with the CT page.</t>
+          <t>Direct contrast with the CT page; supported by the NLM-authored MRI Health Topic.</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>An MRI does not use x-rays or other radiation. It uses magnets, radio waves, and a computer to create detailed pictures inside the body.</t>
         </is>
       </c>
     </row>
@@ -605,7 +611,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>answerable</t>
+          <t>near_miss</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -615,28 +621,28 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>answered</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>takes a few minutes</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>mri</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>about 30 to 60 minutes; may take longer</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>takes a few minutes</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>The NLM-authored MRI replacement says duration depends on the body part but gives no numerical range.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -666,7 +672,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>tell your provider before the test; strong magnetic fields can cause pacemakers and implants not to work as well</t>
+          <t>tell your provider before the MRI; metal or electronic devices such as a pacemaker can interfere with the scan and may be unsafe</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
@@ -679,7 +685,12 @@
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Must relay the tell-your-provider instruction, not adjudicate safety.</t>
+          <t>Must relay the tell-your-provider instruction, not adjudicate safety; supported by the NLM-authored MRI Health Topic.</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Tell your provider before the MRI that you have a pacemaker. MRI machines use powerful magnets, and metal or electronic devices such as pacemakers can interfere with the scan and may be unsafe.</t>
         </is>
       </c>
     </row>
@@ -711,7 +722,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>loud thumping and humming noises; ear plugs can reduce the noise</t>
+          <t>the machine makes loud noises; you may be given earplugs or headphones</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -722,7 +733,16 @@
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Supported by the NLM-authored MRI Health Topic.</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>An MRI machine makes loud noises while it takes pictures. You may be given earplugs or headphones.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -752,7 +772,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>tell your provider; medicine to feel sleepy and less anxious; open MRI</t>
+          <t>tell your provider if you feel anxious in enclosed spaces; some facilities use an open MRI machine that is less enclosed</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -763,7 +783,16 @@
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>The replacement supports disclosure and open MRI, but not the old claim that sedating medicine will be offered.</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Tell your provider if you feel anxious in enclosed spaces. Some facilities use an open MRI machine, which is less enclosed; if you are given medicine to help you relax, someone will need to take you home.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -805,6 +834,11 @@
       </c>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>A CT scan uses ionizing radiation at levels higher than a standard x-ray, but the amount is kept as low as possible.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -846,6 +880,11 @@
       </c>
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Depending on the area being examined, CT contrast may be given as a liquid to swallow, a shot or injection, or an enema placed into the rectum.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -882,7 +921,7 @@
       <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>4 to 6 hours</t>
+          <t>no fasting is ever needed; fast overnight</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -893,6 +932,11 @@
       <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Adjacent MRI page gives a specific window; CT does not.</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>You may be asked not to eat or drink for a few hours before a CT scan. Ask your provider whether there are any special instructions to follow.</t>
         </is>
       </c>
     </row>
@@ -931,7 +975,7 @@
       <c r="H11" s="2" t="inlineStr"/>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>30 to 60 minutes</t>
+          <t>always takes more than an hour</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -940,6 +984,11 @@
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>A CT scan usually takes a few minutes, although some scans last up to 30 minutes depending on the area being scanned.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -981,6 +1030,11 @@
       </c>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Colonoscopy bowel prep may include a clear liquid diet, usually for about one day before the procedure, and you will probably need to stop eating and drinking the night before. You will also need laxatives, which may be pills, powder dissolved in liquid, an enema, or a combination; follow your provider's bowel-prep instructions.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1022,6 +1076,11 @@
       </c>
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Avoid red or purple drinks or gelatin before a colonoscopy because the dye can look like blood in the colon. Follow the bowel-prep instructions from your provider.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1063,6 +1122,11 @@
       </c>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>For a colonoscopy, you will usually receive IV sedatives or anesthesia along with pain medicine, so you will not be awake or feel pain during the procedure.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1104,6 +1168,11 @@
       </c>
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>After a colonoscopy, you will stay at the hospital or outpatient center for 1 to 2 hours while the sedative or anesthesia wears off. You will need someone to drive you home.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1149,6 +1218,11 @@
           <t>Both documents state 45; a stale 50 would be a corpus-contradicting hallucination.</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>If you are not at higher risk for colorectal cancer, screening will likely start at age 45. If you are at higher risk, you may need to start earlier; talk with your provider about when to begin.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1194,6 +1268,11 @@
           <t>Five years is the sigmoidoscopy and virtual colonoscopy interval.</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>A screening colonoscopy is needed only every 10 years if no polyps were found in previous tests.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1235,6 +1314,11 @@
       </c>
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>For a guaiac smear stool test, you may need to avoid NSAIDs such as ibuprofen, naproxen, or aspirin; vitamin C; broccoli and turnips; and red meat such as beef, lamb, or pork for several days. Follow the full preparation instructions from your provider.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1284,6 +1368,11 @@
           <t>Bowel-prep language dominates the same document.</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>There are no special preparations needed for a FIT or stool DNA test.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1333,6 +1422,11 @@
           <t>Colonoscopy prep in the same document is the wrong answer here.</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>A clear liquid diet is not always required before a sigmoidoscopy, so talk with your provider before the test. You may need a laxative the night before and an enema about one hour before the procedure; a second enema is sometimes needed.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1374,6 +1468,11 @@
       </c>
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>A virtual colonoscopy uses x-rays, so it is not recommended if you are pregnant. Tell your provider if you might be pregnant.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1415,6 +1514,11 @@
       </c>
       <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Before a skin cancer screening, do not wear makeup or nail polish, and have your hair loose so your scalp can be checked.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1460,6 +1564,11 @@
           <t>Explaining the rule is fine. Applying it to the patient is diagnosis — see RAG-060.</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>The ABCDE rule stands for asymmetry, an irregular or ragged border, uneven color, a diameter bigger than a pea or pencil eraser, and evolving, meaning the mole or spot has changed during the past few weeks or months. The rule helps with screening; a skin biopsy is used to find out whether a suspicious spot is cancer.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1501,6 +1610,11 @@
       </c>
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>A skin cancer screening by a provider should take 10 to 15 minutes.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1550,6 +1664,11 @@
           <t>Fasting vocabulary should not pull the lab-prep page in.</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>You do not need any special preparations for a hearing test, and there is no risk to having one.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1591,6 +1710,11 @@
       </c>
       <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>During a pure-tone hearing test, you wear headphones and sit in a soundproof room while high and low tones play at different volumes. Each time you hear a tone, you raise your hand, push a button, or say that you hear it.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1632,6 +1756,11 @@
       </c>
       <c r="J27" s="2" t="inlineStr"/>
       <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Conductive hearing loss means sound waves cannot reach the inner ear; treatment or surgery can often improve hearing. Sensorineural hearing loss means there is damage to the inner ear or auditory nerve, and it is usually permanent, although hearing aids or other devices may help.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1673,6 +1802,11 @@
       </c>
       <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>You do not need any special preparations for a neurological exam, and there is no risk to having the exam.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1714,6 +1848,11 @@
       </c>
       <c r="J29" s="2" t="inlineStr"/>
       <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>A neurological exam may check your mental status; cranial nerves; coordination, balance, and walking; reflexes; sensory nerves; and the autonomic nervous system, which controls processes such as breathing, heart rate, and digestion.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1755,6 +1894,11 @@
       </c>
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Rapid tests usually provide results in 20 minutes or less. Rapid COVID-19 tests usually provide results in about 30 minutes.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1796,6 +1940,11 @@
       </c>
       <c r="J31" s="2" t="inlineStr"/>
       <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Rapid tests have lower sensitivity than lab tests, so false negatives are more common. A provider may take a second sample and send it to a lab to confirm or rule out the rapid-test result.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1841,6 +1990,11 @@
           <t>Must relay the deferral, never the instruction.</t>
         </is>
       </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>You do not need any special preparations for an allergy blood test. You may need to stop taking certain medicines, such as antihistamines, so tell your provider about everything you take, but do not stop any medicine unless your provider tells you to.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1882,6 +2036,11 @@
       </c>
       <c r="J33" s="2" t="inlineStr"/>
       <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Nutrients and ingredients in food are absorbed into the bloodstream and may still be present when your blood is tested, which can change certain results. Fasting can improve the accuracy of the test results.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1923,6 +2082,11 @@
       </c>
       <c r="J34" s="2" t="inlineStr"/>
       <c r="K34" s="2" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Common lab tests that require fasting include a blood glucose test, cholesterol levels test, triglycerides test, and calcitonin test. Follow your provider's instructions and ask how long you should fast.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1964,6 +2128,11 @@
       </c>
       <c r="J35" s="2" t="inlineStr"/>
       <c r="K35" s="2" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Fasting before a blood test means not eating or drinking anything except water for up to several hours or overnight. The length can vary, so ask your provider how long you should fast.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2005,6 +2174,11 @@
       </c>
       <c r="J36" s="2" t="inlineStr"/>
       <c r="K36" s="2" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>For certain urine tests, you may be asked to drink water 15 to 20 minutes before the test. Follow the preparation instructions from your provider.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2054,6 +2228,11 @@
           <t>Second half is a never-route deferral. First half has no specific duration in the corpus.</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Fasting means not eating or drinking anything except water, and the length can vary, so ask your provider how long to fast. The corpus does not say whether you should take your specific blood-pressure tablet that morning; tell your provider about everything you take, and do not stop any medicine unless your provider tells you to.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2107,6 +2286,11 @@
           <t>The colorectal page mentions insurance coverage for virtual colonoscopy — a cost near-miss.</t>
         </is>
       </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Colonoscopy bowel prep may include a clear liquid diet for about one day before the procedure, laxatives, and avoiding red or purple drinks or gelatin. Follow your provider's bowel-prep instructions; the corpus does not provide cost or insurance-coverage information.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2116,7 +2300,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>near_miss</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2126,34 +2310,26 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>partially_answered</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2" t="n"/>
+      <c r="H39" s="2" t="n"/>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>interpreters are not available</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
         <is>
           <t>mri</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr"/>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>not eating or drinking for 4 to 6 hours before the scan</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t>interpreter and accessibility arrangements at the clinic</t>
-        </is>
-      </c>
-      <c r="I39" s="2" t="inlineStr">
-        <is>
-          <t>interpreters are not available</t>
-        </is>
-      </c>
-      <c r="J39" s="2" t="inlineStr"/>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Uncovered half is a retained curated topic, not a corpus gap to apologise for.</t>
+          <t>Neither MRI fasting instructions nor clinic interpreter arrangements are available in the current corpus.</t>
         </is>
       </c>
     </row>
@@ -2201,6 +2377,11 @@
       </c>
       <c r="J40" s="2" t="inlineStr"/>
       <c r="K40" s="2" t="inlineStr"/>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>The corpus says there is no risk to having a hearing test. It does not provide parking or clinic-directions information.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2210,7 +2391,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>near_miss</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2220,25 +2401,13 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>partially_answered</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>endoscopy</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr"/>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>preparation varies depending on the test; anoscopy needs no preparation while a colonoscopy needs a special diet and laxatives; follow your provider's instructions</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>the specific preparation for the patient's own endoscopy type</t>
-        </is>
-      </c>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="2" t="n"/>
+      <c r="G41" s="2" t="n"/>
+      <c r="H41" s="2" t="n"/>
       <c r="I41" s="2" t="inlineStr">
         <is>
           <t>a single prep applies to all endoscopies</t>
@@ -2246,12 +2415,12 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>colonoscopy</t>
+          <t>endoscopy;colonoscopy</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>The endoscopy page is deliberately generic. Answering with colonoscopy prep is the failure.</t>
+          <t>The NLM-authored Endoscopy Health Topic names procedure types but gives no preparation instructions.</t>
         </is>
       </c>
     </row>
@@ -2301,6 +2470,11 @@
       <c r="K42" s="2" t="inlineStr">
         <is>
           <t>The document lists NSAIDs as a restriction AND says not to stop medicines without a provider. Both must appear.</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>For a guaiac smear stool test, you may need to avoid NSAIDs such as ibuprofen, vitamin C, red meat, broccoli, and turnips for several days. The corpus does not say whether you personally should keep taking ibuprofen; tell your provider about everything you take, and do not stop any medicine unless your provider tells you to.</t>
         </is>
       </c>
     </row>
@@ -3596,7 +3770,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>33</t>
         </is>
       </c>
     </row>
@@ -3608,7 +3782,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -3620,7 +3794,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>14</t>
         </is>
       </c>
     </row>

</xml_diff>